<commit_message>
refactor: consolidar documentacion HTML de profesorado y alumnado
</commit_message>
<xml_diff>
--- a/profesorado/evaluacion/ponderacionRaCEyCriterios.xlsx
+++ b/profesorado/evaluacion/ponderacionRaCEyCriterios.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Ponderacion por RA" sheetId="1" state="visible" r:id="rId3"/>
@@ -106,7 +106,7 @@
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">VigiaSenior · Ponderación interna de criterios por RA</t>
+    <t xml:space="preserve">VigiaSenior · Ponderación de criterios por RA</t>
   </si>
   <si>
     <t xml:space="preserve">Criterio / agrupación</t>
@@ -675,6 +675,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -731,6 +732,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="10">
@@ -944,232 +946,236 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="5" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="5" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="6" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="7" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="8" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="9" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="9" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="9" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="9" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="9" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="9" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="9" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="9" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="5" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="5" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="6" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="7" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="8" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="9" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="9" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1524,134 +1530,134 @@
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="74.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="50.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="74.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="50.08"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="7" t="n">
+      <c r="C3" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="15" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="15" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="15" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="20" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20"/>
-      <c r="B8" s="21" t="s">
+      <c r="A8" s="21"/>
+      <c r="B8" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="D8" s="21"/>
-      <c r="E8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1678,621 +1684,621 @@
   <dimension ref="A1:F31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="31.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="31.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="46.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="31.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="31.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="34.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="46.61"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="26" t="n">
+      <c r="D3" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="E3" s="26" t="n">
+      <c r="E3" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="F3" s="27" t="s">
+      <c r="F3" s="28" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="30" t="n">
+      <c r="D4" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="E4" s="30" t="n">
+      <c r="E4" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="F4" s="31" t="s">
+      <c r="F4" s="32" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="30" t="n">
+      <c r="D5" s="31" t="n">
         <v>40</v>
       </c>
-      <c r="E5" s="30" t="n">
+      <c r="E5" s="31" t="n">
         <v>8</v>
       </c>
-      <c r="F5" s="31" t="s">
+      <c r="F5" s="32" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="30" t="n">
+      <c r="D6" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="E6" s="30" t="n">
+      <c r="E6" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="31" t="s">
+      <c r="F6" s="32" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="D7" s="30" t="n">
+      <c r="D7" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="31" t="s">
+      <c r="F7" s="32" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="33" t="s">
+      <c r="C8" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="D8" s="34" t="n">
+      <c r="D8" s="35" t="n">
         <v>10</v>
       </c>
-      <c r="E8" s="34" t="n">
+      <c r="E8" s="35" t="n">
         <v>2.5</v>
       </c>
-      <c r="F8" s="35" t="s">
+      <c r="F8" s="36" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="34" t="n">
+      <c r="D9" s="35" t="n">
         <v>15</v>
       </c>
-      <c r="E9" s="34" t="n">
+      <c r="E9" s="35" t="n">
         <v>3.75</v>
       </c>
-      <c r="F9" s="35" t="s">
+      <c r="F9" s="36" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="D10" s="34" t="n">
+      <c r="D10" s="35" t="n">
         <v>20</v>
       </c>
-      <c r="E10" s="34" t="n">
+      <c r="E10" s="35" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="35" t="s">
+      <c r="F10" s="36" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="C11" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="34" t="n">
+      <c r="D11" s="35" t="n">
         <v>15</v>
       </c>
-      <c r="E11" s="34" t="n">
+      <c r="E11" s="35" t="n">
         <v>3.75</v>
       </c>
-      <c r="F11" s="35" t="s">
+      <c r="F11" s="36" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="32" t="s">
+      <c r="A12" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="C12" s="33" t="s">
+      <c r="C12" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="D12" s="34" t="n">
+      <c r="D12" s="35" t="n">
         <v>20</v>
       </c>
-      <c r="E12" s="34" t="n">
+      <c r="E12" s="35" t="n">
         <v>5</v>
       </c>
-      <c r="F12" s="35" t="s">
+      <c r="F12" s="36" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="C13" s="33" t="s">
+      <c r="C13" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="34" t="n">
+      <c r="D13" s="35" t="n">
         <v>20</v>
       </c>
-      <c r="E13" s="34" t="n">
+      <c r="E13" s="35" t="n">
         <v>5</v>
       </c>
-      <c r="F13" s="35" t="s">
+      <c r="F13" s="36" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="36" t="s">
+      <c r="A14" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="37" t="s">
+      <c r="B14" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="C14" s="37" t="s">
+      <c r="C14" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="D14" s="38" t="n">
+      <c r="D14" s="39" t="n">
         <v>10</v>
       </c>
-      <c r="E14" s="38" t="n">
+      <c r="E14" s="39" t="n">
         <v>2.5</v>
       </c>
-      <c r="F14" s="39" t="s">
+      <c r="F14" s="40" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="36" t="s">
+      <c r="A15" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="37" t="s">
+      <c r="B15" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="37" t="s">
+      <c r="C15" s="38" t="s">
         <v>67</v>
       </c>
-      <c r="D15" s="38" t="n">
+      <c r="D15" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="E15" s="38" t="n">
+      <c r="E15" s="39" t="n">
         <v>3.75</v>
       </c>
-      <c r="F15" s="39" t="s">
+      <c r="F15" s="40" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="36" t="s">
+      <c r="A16" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="37" t="s">
+      <c r="B16" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="C16" s="37" t="s">
+      <c r="C16" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="D16" s="38" t="n">
+      <c r="D16" s="39" t="n">
         <v>25</v>
       </c>
-      <c r="E16" s="38" t="n">
+      <c r="E16" s="39" t="n">
         <v>6.25</v>
       </c>
-      <c r="F16" s="39" t="s">
+      <c r="F16" s="40" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="37" t="s">
+      <c r="B17" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="37" t="s">
+      <c r="C17" s="38" t="s">
         <v>71</v>
       </c>
-      <c r="D17" s="38" t="n">
+      <c r="D17" s="39" t="n">
         <v>20</v>
       </c>
-      <c r="E17" s="38" t="n">
+      <c r="E17" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="F17" s="39" t="s">
+      <c r="F17" s="40" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="36" t="s">
+      <c r="A18" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="37" t="s">
+      <c r="B18" s="38" t="s">
         <v>73</v>
       </c>
-      <c r="C18" s="37" t="s">
+      <c r="C18" s="38" t="s">
         <v>74</v>
       </c>
-      <c r="D18" s="38" t="n">
+      <c r="D18" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="E18" s="38" t="n">
+      <c r="E18" s="39" t="n">
         <v>3.75</v>
       </c>
-      <c r="F18" s="39" t="s">
+      <c r="F18" s="40" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="36" t="s">
+      <c r="A19" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="37" t="s">
+      <c r="B19" s="38" t="s">
         <v>76</v>
       </c>
-      <c r="C19" s="37" t="s">
+      <c r="C19" s="38" t="s">
         <v>77</v>
       </c>
-      <c r="D19" s="38" t="n">
+      <c r="D19" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="E19" s="38" t="n">
+      <c r="E19" s="39" t="n">
         <v>3.75</v>
       </c>
-      <c r="F19" s="39" t="s">
+      <c r="F19" s="40" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="40" t="s">
+      <c r="A20" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="41" t="s">
+      <c r="B20" s="42" t="s">
         <v>79</v>
       </c>
-      <c r="C20" s="41" t="s">
+      <c r="C20" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="D20" s="42" t="n">
+      <c r="D20" s="43" t="n">
         <v>15</v>
       </c>
-      <c r="E20" s="42" t="n">
+      <c r="E20" s="43" t="n">
         <v>2.25</v>
       </c>
-      <c r="F20" s="43" t="s">
+      <c r="F20" s="44" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="40" t="s">
+      <c r="A21" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="41" t="s">
+      <c r="B21" s="42" t="s">
         <v>82</v>
       </c>
-      <c r="C21" s="41" t="s">
+      <c r="C21" s="42" t="s">
         <v>83</v>
       </c>
-      <c r="D21" s="42" t="n">
+      <c r="D21" s="43" t="n">
         <v>25</v>
       </c>
-      <c r="E21" s="42" t="n">
+      <c r="E21" s="43" t="n">
         <v>3.75</v>
       </c>
-      <c r="F21" s="43" t="s">
+      <c r="F21" s="44" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="41" t="s">
+      <c r="B22" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="C22" s="41" t="s">
+      <c r="C22" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="D22" s="42" t="n">
+      <c r="D22" s="43" t="n">
         <v>20</v>
       </c>
-      <c r="E22" s="42" t="n">
+      <c r="E22" s="43" t="n">
         <v>3</v>
       </c>
-      <c r="F22" s="43" t="s">
+      <c r="F22" s="44" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="40" t="s">
+      <c r="A23" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="41" t="s">
+      <c r="B23" s="42" t="s">
         <v>87</v>
       </c>
-      <c r="C23" s="41" t="s">
+      <c r="C23" s="42" t="s">
         <v>88</v>
       </c>
-      <c r="D23" s="42" t="n">
+      <c r="D23" s="43" t="n">
         <v>20</v>
       </c>
-      <c r="E23" s="42" t="n">
+      <c r="E23" s="43" t="n">
         <v>3</v>
       </c>
-      <c r="F23" s="43" t="s">
+      <c r="F23" s="44" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="40" t="s">
+      <c r="A24" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="41" t="s">
+      <c r="B24" s="42" t="s">
         <v>89</v>
       </c>
-      <c r="C24" s="41" t="s">
+      <c r="C24" s="42" t="s">
         <v>90</v>
       </c>
-      <c r="D24" s="42" t="n">
+      <c r="D24" s="43" t="n">
         <v>20</v>
       </c>
-      <c r="E24" s="42" t="n">
+      <c r="E24" s="43" t="n">
         <v>3</v>
       </c>
-      <c r="F24" s="43" t="s">
+      <c r="F24" s="44" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="44" t="s">
+      <c r="A25" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="45" t="s">
+      <c r="B25" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="C25" s="45" t="s">
+      <c r="C25" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="D25" s="46" t="n">
+      <c r="D25" s="47" t="n">
         <v>10</v>
       </c>
-      <c r="E25" s="46" t="n">
+      <c r="E25" s="47" t="n">
         <v>1.5</v>
       </c>
-      <c r="F25" s="47" t="s">
+      <c r="F25" s="48" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="44" t="s">
+      <c r="A26" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="45" t="s">
+      <c r="B26" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="C26" s="45" t="s">
+      <c r="C26" s="46" t="s">
         <v>95</v>
       </c>
-      <c r="D26" s="46" t="n">
+      <c r="D26" s="47" t="n">
         <v>15</v>
       </c>
-      <c r="E26" s="46" t="n">
+      <c r="E26" s="47" t="n">
         <v>2.25</v>
       </c>
-      <c r="F26" s="47" t="s">
+      <c r="F26" s="48" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="44" t="s">
+      <c r="A27" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="45" t="s">
+      <c r="B27" s="46" t="s">
         <v>97</v>
       </c>
-      <c r="C27" s="45" t="s">
+      <c r="C27" s="46" t="s">
         <v>98</v>
       </c>
-      <c r="D27" s="46" t="n">
+      <c r="D27" s="47" t="n">
         <v>20</v>
       </c>
-      <c r="E27" s="46" t="n">
+      <c r="E27" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="F27" s="47" t="s">
+      <c r="F27" s="48" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="44" t="s">
+      <c r="A28" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="45" t="s">
+      <c r="B28" s="46" t="s">
         <v>99</v>
       </c>
-      <c r="C28" s="45" t="s">
+      <c r="C28" s="46" t="s">
         <v>100</v>
       </c>
-      <c r="D28" s="46" t="n">
+      <c r="D28" s="47" t="n">
         <v>15</v>
       </c>
-      <c r="E28" s="46" t="n">
+      <c r="E28" s="47" t="n">
         <v>2.25</v>
       </c>
-      <c r="F28" s="47" t="s">
+      <c r="F28" s="48" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="44" t="s">
+      <c r="A29" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="B29" s="45" t="s">
+      <c r="B29" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="C29" s="45" t="s">
+      <c r="C29" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="D29" s="46" t="n">
+      <c r="D29" s="47" t="n">
         <v>15</v>
       </c>
-      <c r="E29" s="46" t="n">
+      <c r="E29" s="47" t="n">
         <v>2.25</v>
       </c>
-      <c r="F29" s="47" t="s">
+      <c r="F29" s="48" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="44" t="s">
+      <c r="A30" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="B30" s="45" t="s">
+      <c r="B30" s="46" t="s">
         <v>104</v>
       </c>
-      <c r="C30" s="45" t="s">
+      <c r="C30" s="46" t="s">
         <v>105</v>
       </c>
-      <c r="D30" s="46" t="n">
+      <c r="D30" s="47" t="n">
         <v>10</v>
       </c>
-      <c r="E30" s="46" t="n">
+      <c r="E30" s="47" t="n">
         <v>1.5</v>
       </c>
-      <c r="F30" s="47" t="s">
+      <c r="F30" s="48" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="48" t="s">
+      <c r="A31" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="B31" s="49" t="s">
+      <c r="B31" s="50" t="s">
         <v>106</v>
       </c>
-      <c r="C31" s="49" t="s">
+      <c r="C31" s="50" t="s">
         <v>107</v>
       </c>
-      <c r="D31" s="50" t="n">
+      <c r="D31" s="51" t="n">
         <v>15</v>
       </c>
-      <c r="E31" s="50" t="n">
+      <c r="E31" s="51" t="n">
         <v>2.25</v>
       </c>
-      <c r="F31" s="51" t="s">
+      <c r="F31" s="52" t="s">
         <v>78</v>
       </c>
     </row>
@@ -2321,312 +2327,312 @@
   <dimension ref="A1:K12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="53" t="s">
         <v>109</v>
       </c>
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="54" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="53" t="s">
+      <c r="C2" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D2" s="53" t="s">
+      <c r="D2" s="54" t="s">
         <v>112</v>
       </c>
-      <c r="E2" s="53" t="s">
+      <c r="E2" s="54" t="s">
         <v>113</v>
       </c>
-      <c r="F2" s="53" t="s">
+      <c r="F2" s="54" t="s">
         <v>114</v>
       </c>
-      <c r="G2" s="53" t="s">
+      <c r="G2" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="54" t="s">
+      <c r="H2" s="55" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="G3" s="7" t="n">
+      <c r="G3" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="10" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="G4" s="12" t="n">
+      <c r="G4" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="15" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="H5" s="15" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="H6" s="14" t="s">
+      <c r="H6" s="15" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="15" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="15" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="G9" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="H9" s="15" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="14" t="s">
         <v>155</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="H10" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="K10" s="55"/>
+      <c r="K10" s="56"/>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="14" t="s">
         <v>160</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="G11" s="12" t="n">
+      <c r="G11" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="H11" s="15" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>164</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="19" t="s">
         <v>166</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="G12" s="17" t="n">
+      <c r="G12" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="H12" s="56" t="s">
+      <c r="H12" s="57" t="s">
         <v>169</v>
       </c>
     </row>
@@ -2667,160 +2673,160 @@
   <dimension ref="A1:G1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="28"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="53" t="s">
         <v>171</v>
       </c>
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="54" t="s">
         <v>172</v>
       </c>
-      <c r="C2" s="53" t="s">
+      <c r="C2" s="54" t="s">
         <v>173</v>
       </c>
-      <c r="D2" s="53" t="s">
+      <c r="D2" s="54" t="s">
         <v>174</v>
       </c>
-      <c r="E2" s="53" t="s">
+      <c r="E2" s="54" t="s">
         <v>175</v>
       </c>
-      <c r="F2" s="53" t="s">
+      <c r="F2" s="54" t="s">
         <v>176</v>
       </c>
-      <c r="G2" s="54" t="s">
+      <c r="G2" s="55" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="10" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="11" t="s">
         <v>185</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="14" t="s">
         <v>189</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="15" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="14" t="s">
         <v>197</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="15" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="11" t="s">
         <v>199</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="14" t="s">
         <v>201</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="14" t="s">
         <v>202</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="14" t="s">
         <v>203</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G6" s="15" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="16" t="s">
         <v>205</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="20" t="s">
         <v>211</v>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: pulir RA/CE en xlsx
</commit_message>
<xml_diff>
--- a/profesorado/evaluacion/ponderacionRaCEyCriterios.xlsx
+++ b/profesorado/evaluacion/ponderacionRaCEyCriterios.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Ponderacion por RA" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="210">
   <si>
     <t xml:space="preserve">VigiaSenior · Ponderación global de la evaluación por resultados de aprendizaje</t>
   </si>
@@ -253,102 +253,96 @@
     <t xml:space="preserve">Sesiones 8-9</t>
   </si>
   <si>
-    <t xml:space="preserve">7.h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documentación del servicio</t>
+    <t xml:space="preserve">8.c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tecnologías y frameworks relacionados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sesión 4-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación de datos con interacción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sesión 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validación de entradas o formularios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modificación dinámica de contenido y estructura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aplicación de estas tecnologías al proyecto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reutilización de código e información</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sesiones 5-9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tecnologías o frameworks aplicables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sesiones 4-9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recuperación y procesamiento de información existente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Creación de repositorios o estructuras derivadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sesiones 6-9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incorporación de funcionalidades específicas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uso de servicios o código de terceros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pruebas, depuración y documentación</t>
   </si>
   <si>
     <t xml:space="preserve">Sesiones 9-10</t>
   </si>
   <si>
-    <t xml:space="preserve">8.c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tecnologías y frameworks relacionados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sesión 4-8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.d</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación de datos con interacción</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sesión 8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validación de entradas o formularios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.f</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modificación dinámica de contenido y estructura</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aplicación de estas tecnologías al proyecto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reutilización de código e información</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sesiones 5-9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tecnologías o frameworks aplicables</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sesiones 4-9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recuperación y procesamiento de información existente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.d</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Creación de repositorios o estructuras derivadas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sesiones 6-9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Incorporación de funcionalidades específicas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.f</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uso de servicios o código de terceros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pruebas, depuración y documentación</t>
-  </si>
-  <si>
     <t xml:space="preserve">VigiaSenior · Evidencias, instrumentos y momento de utilización</t>
   </si>
   <si>
@@ -490,10 +484,10 @@
     <t xml:space="preserve">Sesión 9 · Hito 3</t>
   </si>
   <si>
-    <t xml:space="preserve">9.b, 9.c, 9.e, 9.h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pruebas sobre el simulador o el modelo de pruebas fisico.</t>
+    <t xml:space="preserve">9.b, 9.c, 9.e, 9.g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pruebas sobre el simulador o el modelo de pruebas físico</t>
   </si>
   <si>
     <t xml:space="preserve">Documentación técnica y organización del repositorio</t>
@@ -505,7 +499,7 @@
     <t xml:space="preserve">RA5, RA6, RA7, RA9</t>
   </si>
   <si>
-    <t xml:space="preserve">5.h, 6.g, 7.h, 9.h</t>
+    <t xml:space="preserve">5.h, 6.g, 9.g</t>
   </si>
   <si>
     <t xml:space="preserve">Rúbrica documental</t>
@@ -520,10 +514,10 @@
     <t xml:space="preserve">Sesión 10 · Cierre</t>
   </si>
   <si>
-    <t xml:space="preserve">Transversal + proyecto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comunicación, justificación y síntesis</t>
+    <t xml:space="preserve">RA5, RA6, RA7, RA8, RA9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.g, 5.h, 6.b, 6.c, 6.d, 7.e, 7.f, 7.g, 8.g, 9.b, 9.c, 9.e</t>
   </si>
   <si>
     <t xml:space="preserve">Rúbrica de presentación</t>
@@ -532,7 +526,7 @@
     <t xml:space="preserve">Equipo (con reparto individual)</t>
   </si>
   <si>
-    <t xml:space="preserve">Participación de ambos miembros en la defensa oral, con reparto claro de contenidos, equilibrio en el tiempo de intervención y coherencia expositiva.</t>
+    <t xml:space="preserve">Se valora la capacidad de explicar las decisiones técnicas del proyecto, justificar el diseño adoptado, defender el funcionamiento del backend y sintetizar el proceso seguido, con participación equilibrada de los miembros del equipo.</t>
   </si>
   <si>
     <t xml:space="preserve">VigiaSenior · Calendario de sesiones, hitos y entregas</t>
@@ -670,7 +664,7 @@
     <numFmt numFmtId="165" formatCode="0"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -731,6 +725,12 @@
       <u val="single"/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
@@ -946,7 +946,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1173,6 +1173,10 @@
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1356,7 +1360,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CriteriosRA" displayName="CriteriosRA" ref="A2:F31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CriteriosRA" displayName="CriteriosRA" ref="A2:F30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="6">
     <tableColumn id="1" name="RA"/>
     <tableColumn id="2" name="Criterio / agrupación"/>
@@ -1681,7 +1685,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
@@ -1953,10 +1957,10 @@
         <v>64</v>
       </c>
       <c r="D14" s="39" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E14" s="39" t="n">
-        <v>2.5</v>
+        <v>3.75</v>
       </c>
       <c r="F14" s="40" t="s">
         <v>65</v>
@@ -1973,10 +1977,10 @@
         <v>67</v>
       </c>
       <c r="D15" s="39" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E15" s="39" t="n">
-        <v>3.75</v>
+        <v>5</v>
       </c>
       <c r="F15" s="40" t="s">
         <v>65</v>
@@ -2033,32 +2037,32 @@
         <v>74</v>
       </c>
       <c r="D18" s="39" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E18" s="39" t="n">
-        <v>3.75</v>
+        <v>5</v>
       </c>
       <c r="F18" s="40" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="37" t="s">
-        <v>14</v>
-      </c>
-      <c r="B19" s="38" t="s">
+      <c r="A19" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="42" t="s">
         <v>76</v>
       </c>
-      <c r="C19" s="38" t="s">
+      <c r="C19" s="42" t="s">
         <v>77</v>
       </c>
-      <c r="D19" s="39" t="n">
+      <c r="D19" s="43" t="n">
         <v>15</v>
       </c>
-      <c r="E19" s="39" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="F19" s="40" t="s">
+      <c r="E19" s="43" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F19" s="44" t="s">
         <v>78</v>
       </c>
     </row>
@@ -2073,10 +2077,10 @@
         <v>80</v>
       </c>
       <c r="D20" s="43" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E20" s="43" t="n">
-        <v>2.25</v>
+        <v>3.75</v>
       </c>
       <c r="F20" s="44" t="s">
         <v>81</v>
@@ -2093,24 +2097,24 @@
         <v>83</v>
       </c>
       <c r="D21" s="43" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E21" s="43" t="n">
-        <v>3.75</v>
+        <v>3</v>
       </c>
       <c r="F21" s="44" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="41" t="s">
         <v>18</v>
       </c>
       <c r="B22" s="42" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" s="42" t="s">
         <v>85</v>
-      </c>
-      <c r="C22" s="42" t="s">
-        <v>86</v>
       </c>
       <c r="D22" s="43" t="n">
         <v>20</v>
@@ -2119,18 +2123,18 @@
         <v>3</v>
       </c>
       <c r="F22" s="44" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="41" t="s">
         <v>18</v>
       </c>
       <c r="B23" s="42" t="s">
+        <v>86</v>
+      </c>
+      <c r="C23" s="42" t="s">
         <v>87</v>
-      </c>
-      <c r="C23" s="42" t="s">
-        <v>88</v>
       </c>
       <c r="D23" s="43" t="n">
         <v>20</v>
@@ -2139,27 +2143,27 @@
         <v>3</v>
       </c>
       <c r="F23" s="44" t="s">
-        <v>84</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="B24" s="42" t="s">
+      <c r="A24" s="45" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" s="46" t="s">
+        <v>88</v>
+      </c>
+      <c r="C24" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="C24" s="42" t="s">
+      <c r="D24" s="47" t="n">
+        <v>10</v>
+      </c>
+      <c r="E24" s="47" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F24" s="48" t="s">
         <v>90</v>
-      </c>
-      <c r="D24" s="43" t="n">
-        <v>20</v>
-      </c>
-      <c r="E24" s="43" t="n">
-        <v>3</v>
-      </c>
-      <c r="F24" s="44" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2173,16 +2177,16 @@
         <v>92</v>
       </c>
       <c r="D25" s="47" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E25" s="47" t="n">
-        <v>1.5</v>
+        <v>2.25</v>
       </c>
       <c r="F25" s="48" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="45" t="s">
         <v>22</v>
       </c>
@@ -2193,13 +2197,13 @@
         <v>95</v>
       </c>
       <c r="D26" s="47" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E26" s="47" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="F26" s="48" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2207,22 +2211,22 @@
         <v>22</v>
       </c>
       <c r="B27" s="46" t="s">
+        <v>96</v>
+      </c>
+      <c r="C27" s="46" t="s">
         <v>97</v>
       </c>
-      <c r="C27" s="46" t="s">
+      <c r="D27" s="47" t="n">
+        <v>15</v>
+      </c>
+      <c r="E27" s="47" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F27" s="48" t="s">
         <v>98</v>
       </c>
-      <c r="D27" s="47" t="n">
-        <v>20</v>
-      </c>
-      <c r="E27" s="47" t="n">
-        <v>3</v>
-      </c>
-      <c r="F27" s="48" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="45" t="s">
         <v>22</v>
       </c>
@@ -2239,7 +2243,7 @@
         <v>2.25</v>
       </c>
       <c r="F28" s="48" t="s">
-        <v>101</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2247,61 +2251,42 @@
         <v>22</v>
       </c>
       <c r="B29" s="46" t="s">
+        <v>101</v>
+      </c>
+      <c r="C29" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="C29" s="46" t="s">
-        <v>103</v>
-      </c>
       <c r="D29" s="47" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E29" s="47" t="n">
-        <v>2.25</v>
+        <v>1.5</v>
       </c>
       <c r="F29" s="48" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="45" t="s">
+      <c r="A30" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="B30" s="46" t="s">
+      <c r="B30" s="50" t="s">
+        <v>103</v>
+      </c>
+      <c r="C30" s="50" t="s">
         <v>104</v>
       </c>
-      <c r="C30" s="46" t="s">
+      <c r="D30" s="51" t="n">
+        <v>15</v>
+      </c>
+      <c r="E30" s="51" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F30" s="52" t="s">
         <v>105</v>
       </c>
-      <c r="D30" s="47" t="n">
-        <v>10</v>
-      </c>
-      <c r="E30" s="47" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F30" s="48" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="49" t="s">
-        <v>22</v>
-      </c>
-      <c r="B31" s="50" t="s">
-        <v>106</v>
-      </c>
-      <c r="C31" s="50" t="s">
-        <v>107</v>
-      </c>
-      <c r="D31" s="51" t="n">
-        <v>15</v>
-      </c>
-      <c r="E31" s="51" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="F31" s="52" t="s">
-        <v>78</v>
-      </c>
-    </row>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
@@ -2332,14 +2317,14 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="6" min="6" style="1" width="29.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B1" s="24"/>
       <c r="C1" s="24"/>
@@ -2351,289 +2336,289 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="53" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" s="54" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="54" t="s">
         <v>109</v>
       </c>
-      <c r="B2" s="54" t="s">
+      <c r="D2" s="54" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="54" t="s">
+      <c r="E2" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D2" s="54" t="s">
+      <c r="F2" s="54" t="s">
         <v>112</v>
-      </c>
-      <c r="E2" s="54" t="s">
-        <v>113</v>
-      </c>
-      <c r="F2" s="54" t="s">
-        <v>114</v>
       </c>
       <c r="G2" s="54" t="s">
         <v>3</v>
       </c>
       <c r="H2" s="55" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="E3" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="F3" s="9" t="s">
         <v>119</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>121</v>
       </c>
       <c r="G3" s="8" t="n">
         <v>10</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C4" s="14" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G4" s="13" t="n">
         <v>10</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G5" s="13" t="n">
         <v>10</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G6" s="13" t="n">
         <v>10</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>13</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G7" s="13" t="n">
         <v>15</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C8" s="14" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G8" s="13" t="n">
         <v>15</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="C9" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="D9" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="E9" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="D9" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>151</v>
-      </c>
       <c r="F9" s="14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G9" s="13" t="n">
         <v>15</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E10" s="14" t="s">
         <v>25</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G10" s="13" t="n">
         <v>10</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="K10" s="56"/>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="D11" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="E11" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="D11" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>161</v>
-      </c>
       <c r="F11" s="14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G11" s="13" t="n">
         <v>5</v>
       </c>
       <c r="H11" s="15" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="B12" s="19" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="16" t="s">
+      <c r="C12" s="17" t="s">
         <v>163</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="D12" s="57" t="s">
         <v>164</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="E12" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="F12" s="19" t="s">
         <v>166</v>
-      </c>
-      <c r="E12" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="F12" s="19" t="s">
-        <v>168</v>
       </c>
       <c r="G12" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="H12" s="57" t="s">
-        <v>169</v>
+      <c r="H12" s="58" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -2683,7 +2668,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B1" s="24"/>
       <c r="C1" s="24"/>
@@ -2694,140 +2679,140 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="53" t="s">
+        <v>169</v>
+      </c>
+      <c r="B2" s="54" t="s">
+        <v>170</v>
+      </c>
+      <c r="C2" s="54" t="s">
         <v>171</v>
       </c>
-      <c r="B2" s="54" t="s">
+      <c r="D2" s="54" t="s">
         <v>172</v>
       </c>
-      <c r="C2" s="54" t="s">
+      <c r="E2" s="54" t="s">
         <v>173</v>
       </c>
-      <c r="D2" s="54" t="s">
+      <c r="F2" s="54" t="s">
         <v>174</v>
       </c>
-      <c r="E2" s="54" t="s">
+      <c r="G2" s="55" t="s">
         <v>175</v>
-      </c>
-      <c r="F2" s="54" t="s">
-        <v>176</v>
-      </c>
-      <c r="G2" s="55" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="E3" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="F3" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="G3" s="10" t="s">
         <v>182</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="C4" s="14" t="s">
         <v>185</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="D4" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="E4" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="F4" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="G4" s="15" t="s">
         <v>189</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>190</v>
-      </c>
-      <c r="G4" s="15" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="C5" s="14" t="s">
         <v>192</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="D5" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="E5" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="F5" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="G5" s="15" t="s">
         <v>196</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>197</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>199</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="D6" s="14" t="s">
+        <v>193</v>
+      </c>
+      <c r="E6" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="F6" s="14" t="s">
         <v>201</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>195</v>
-      </c>
-      <c r="E6" s="14" t="s">
+      <c r="G6" s="15" t="s">
         <v>202</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>203</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>204</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="D7" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="E7" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="F7" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="G7" s="20" t="s">
         <v>209</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="G7" s="20" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>